<commit_message>
Coal report 20.09.2026 (update 3)
</commit_message>
<xml_diff>
--- a/reports/2026-09-20.xlsx
+++ b/reports/2026-09-20.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D015837D-1BD9-AC46-AF59-ECE15DCF91B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9AFA522A-CE29-8B44-8390-01C8B3101E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6696,7 +6696,7 @@
       <c r="R59" s="60"/>
       <c r="S59" s="60"/>
     </row>
-    <row r="60" spans="1:19" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:19" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="3"/>
       <c r="B60" s="344" t="s">
         <v>249</v>

</xml_diff>